<commit_message>
feat: orderdate added to forms and schemas
</commit_message>
<xml_diff>
--- a/client/public/templates/agendamentos.xlsx
+++ b/client/public/templates/agendamentos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScopeSystem\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC59B6F-634F-470E-8DE8-AB3FAEA5D0E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9EF454-8438-41BF-B810-ED3F1DDC31B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2E23A2F0-7916-498F-87CC-10548E8D6FB9}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
   <si>
     <t>Placa</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>campos da manutenção</t>
+  </si>
+  <si>
+    <t>Data do pedido</t>
   </si>
 </sst>
 </file>
@@ -209,11 +212,8 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
@@ -656,90 +656,84 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39DA93B-0796-4B49-A356-7FE058FFC3E5}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultColWidth="18.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="18.26953125" style="2"/>
+    <col min="1" max="2" width="18.26953125" style="1"/>
+    <col min="3" max="3" width="19.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="16384" width="18.26953125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:19" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="F1" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="G1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="K1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="L1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="M1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="N1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="O1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="14" t="s">
+      <c r="P1" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="P1" s="14" t="s">
+      <c r="Q1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="R1" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="S1" s="12" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
-  <conditionalFormatting sqref="B1">
+  <conditionalFormatting sqref="C1">
     <cfRule type="duplicateValues" dxfId="7" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="8"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:D1">
+  <conditionalFormatting sqref="D1:E1">
     <cfRule type="duplicateValues" dxfId="1" priority="9"/>
     <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
@@ -753,13 +747,13 @@
   <sheetFormatPr defaultRowHeight="31" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="20.81640625" customWidth="1"/>
-    <col min="2" max="2" width="4.7265625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="4.7265625" style="2" customWidth="1"/>
     <col min="3" max="3" width="21.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.7">
-      <c r="A1" s="4"/>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="3"/>
+      <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C1" t="s">
@@ -767,8 +761,8 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.7">
-      <c r="A2" s="5"/>
-      <c r="B2" s="3" t="s">
+      <c r="A2" s="4"/>
+      <c r="B2" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C2" t="s">
@@ -776,8 +770,8 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.7">
-      <c r="A3" s="6"/>
-      <c r="B3" s="3" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C3" t="s">

</xml_diff>

<commit_message>
feat: service table + reason mandatory at maintenence and logic updates
</commit_message>
<xml_diff>
--- a/client/public/templates/agendamentos.xlsx
+++ b/client/public/templates/agendamentos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ScopeSystem\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C9EF454-8438-41BF-B810-ED3F1DDC31B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EA78CD-81C4-44B9-8B63-E4D9D551DC93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{2E23A2F0-7916-498F-87CC-10548E8D6FB9}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="25">
   <si>
     <t>Placa</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>Data do pedido</t>
+  </si>
+  <si>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>motivo obrigatorio para manutenção</t>
   </si>
 </sst>
 </file>
@@ -656,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39DA93B-0796-4B49-A356-7FE058FFC3E5}">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr defaultColWidth="18.26953125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="18.26953125" style="1"/>
@@ -664,7 +670,7 @@
     <col min="4" max="16384" width="18.26953125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>22</v>
       </c>
@@ -716,10 +722,13 @@
       <c r="Q1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="R1" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="S1" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="T1" s="12" t="s">
         <v>7</v>
       </c>
     </row>
@@ -743,7 +752,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{155B8B74-C021-4DE1-8FBB-BA72E6D7B43F}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="31" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="20.81640625" customWidth="1"/>
@@ -751,7 +760,7 @@
     <col min="3" max="3" width="21.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A1" s="3"/>
       <c r="B1" s="2" t="s">
         <v>18</v>
@@ -760,7 +769,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A2" s="4"/>
       <c r="B2" s="2" t="s">
         <v>18</v>
@@ -769,13 +778,16 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.7">
       <c r="A3" s="5"/>
       <c r="B3" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C3" t="s">
         <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>